<commit_message>
test: regenerate the workbooks with the fixed seeds
The every-code workbook now exercises BDAY-FUTURE and the SECTOR
fallback warning (the prior SECTOR seed used a valid OTHER code,
which is silent by design), verified through the real importer; the
rest of the set is regenerated in the same pass so the committed
workbooks all come from one generator run.
</commit_message>
<xml_diff>
--- a/excel/family-import-ALL-ERRORS.xlsx
+++ b/excel/family-import-ALL-ERRORS.xlsx
@@ -117,7 +117,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="517">
   <si>
     <t>FAMILY</t>
   </si>
@@ -227,6 +227,9 @@
     <t>9100005</t>
   </si>
   <si>
+    <t>9100014</t>
+  </si>
+  <si>
     <t>9100006</t>
   </si>
   <si>
@@ -332,6 +335,9 @@
     <t>31-31-2000</t>
   </si>
   <si>
+    <t>01-01-2050</t>
+  </si>
+  <si>
     <t>03-03-1979</t>
   </si>
   <si>
@@ -446,6 +452,9 @@
     <t>09171230007</t>
   </si>
   <si>
+    <t>09171230028</t>
+  </si>
+  <si>
     <t>09171230008</t>
   </si>
   <si>
@@ -503,22 +512,22 @@
     <t>09171230017</t>
   </si>
   <si>
-    <t>09000001232</t>
-  </si>
-  <si>
     <t>09000001269</t>
   </si>
   <si>
+    <t>09000001306</t>
+  </si>
+  <si>
     <t>09171230018</t>
   </si>
   <si>
     <t>09171230019</t>
   </si>
   <si>
-    <t>09000001380</t>
-  </si>
-  <si>
-    <t>09000001454</t>
+    <t>09000001417</t>
+  </si>
+  <si>
+    <t>09000001491</t>
   </si>
   <si>
     <t>Head</t>
@@ -668,6 +677,9 @@
     <t>Nilo</t>
   </si>
   <si>
+    <t>Iris</t>
+  </si>
+  <si>
     <t>Rene</t>
   </si>
   <si>
@@ -779,10 +791,7 @@
     <t>Born Again Christian</t>
   </si>
   <si>
-    <t>Seventh-day Adventist</t>
-  </si>
-  <si>
-    <t>No Religion</t>
+    <t>Bible Baptist</t>
   </si>
   <si>
     <t>E - Elementary</t>
@@ -962,61 +971,64 @@
     <t>OFW</t>
   </si>
   <si>
+    <t>ZZ9</t>
+  </si>
+  <si>
+    <t>SC1, SC2</t>
+  </si>
+  <si>
+    <t>PWD1, PWD3</t>
+  </si>
+  <si>
+    <t>B2, B3, 4PS</t>
+  </si>
+  <si>
+    <t>B2, B3</t>
+  </si>
+  <si>
+    <t>SWPS4, 4PS</t>
+  </si>
+  <si>
+    <t>FA2</t>
+  </si>
+  <si>
+    <t>SP1</t>
+  </si>
+  <si>
+    <t>ZZZ</t>
+  </si>
+  <si>
+    <t>FA6, EDA5</t>
+  </si>
+  <si>
+    <t>Relationships</t>
+  </si>
+  <si>
+    <t>SPOUSE</t>
+  </si>
+  <si>
+    <t>CHILD</t>
+  </si>
+  <si>
+    <t>PARENT</t>
+  </si>
+  <si>
+    <t>SIBLING</t>
+  </si>
+  <si>
+    <t>GRANDPARENT</t>
+  </si>
+  <si>
+    <t>GRANDCHILD</t>
+  </si>
+  <si>
+    <t>IN-LAW</t>
+  </si>
+  <si>
+    <t>RELATIVE</t>
+  </si>
+  <si>
     <t>OTHER</t>
-  </si>
-  <si>
-    <t>SC1, SC2</t>
-  </si>
-  <si>
-    <t>PWD1, PWD3</t>
-  </si>
-  <si>
-    <t>B2, B3, 4PS</t>
-  </si>
-  <si>
-    <t>B2, B3</t>
-  </si>
-  <si>
-    <t>SWPS4, 4PS</t>
-  </si>
-  <si>
-    <t>FA2</t>
-  </si>
-  <si>
-    <t>SP1</t>
-  </si>
-  <si>
-    <t>ZZZ</t>
-  </si>
-  <si>
-    <t>FA6, EDA5</t>
-  </si>
-  <si>
-    <t>Relationships</t>
-  </si>
-  <si>
-    <t>SPOUSE</t>
-  </si>
-  <si>
-    <t>CHILD</t>
-  </si>
-  <si>
-    <t>PARENT</t>
-  </si>
-  <si>
-    <t>SIBLING</t>
-  </si>
-  <si>
-    <t>GRANDPARENT</t>
-  </si>
-  <si>
-    <t>GRANDCHILD</t>
-  </si>
-  <si>
-    <t>IN-LAW</t>
-  </si>
-  <si>
-    <t>RELATIVE</t>
   </si>
   <si>
     <t>Suffixes</t>
@@ -2308,53 +2320,53 @@
         <v>26</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="F3" s="12"/>
       <c r="G3" s="11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I3" s="12" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="J3" s="11" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="K3" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L3" s="12" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="M3" s="12" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="N3" s="12" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="O3" s="12" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="P3" s="12" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="Q3" s="12" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="R3" s="12" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="S3" t="str">
         <f>IF(AND($A3="",$C3="",$D3=""),"",IF($A3="","Missing QR Number",IF($C3="","Missing LastName",IF($D3="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A3,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A3,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -2366,53 +2378,53 @@
         <v>27</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F4" s="12"/>
       <c r="G4" s="11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="N4" s="12" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="O4" s="12" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="P4" s="12" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="Q4" s="12" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="R4" s="12" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="S4" t="str">
         <f>IF(AND($A4="",$C4="",$D4=""),"",IF($A4="","Missing QR Number",IF($C4="","Missing LastName",IF($D4="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A4,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A4,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -2424,49 +2436,49 @@
         <v>28</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="F5" s="12"/>
       <c r="G5" s="11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I5" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="K5" s="12" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="L5" s="12" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="N5" s="12" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="O5" s="12"/>
       <c r="P5" s="12"/>
       <c r="Q5" s="12" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="R5" s="12" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="S5" t="str">
         <f>IF(AND($A5="",$C5="",$D5=""),"",IF($A5="","Missing QR Number",IF($C5="","Missing LastName",IF($D5="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A5,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A5,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -2478,53 +2490,53 @@
         <v>29</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="F6" s="12"/>
       <c r="G6" s="11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I6" s="12" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="K6" s="12" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="L6" s="12" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="M6" s="12" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="N6" s="12" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="O6" s="12" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="P6" s="12" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="Q6" s="12" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="R6" s="12" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="S6" t="str">
         <f>IF(AND($A6="",$C6="",$D6=""),"",IF($A6="","Missing QR Number",IF($C6="","Missing LastName",IF($D6="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A6,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A6,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -2536,49 +2548,49 @@
         <v>29</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="F7" s="12"/>
       <c r="G7" s="11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I7" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J7" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="K7" s="12" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="L7" s="12" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="M7" s="12" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="N7" s="12" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="O7" s="12"/>
       <c r="P7" s="12"/>
       <c r="Q7" s="12" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="R7" s="12" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="S7" t="str">
         <f>IF(AND($A7="",$C7="",$D7=""),"",IF($A7="","Missing QR Number",IF($C7="","Missing LastName",IF($D7="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A7,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A7,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -2590,53 +2602,53 @@
         <v>30</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="F8" s="12"/>
       <c r="G8" s="11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J8" s="11" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L8" s="12" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="N8" s="12" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="O8" s="12" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="P8" s="12" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="Q8" s="12" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="R8" s="12" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="S8" t="str">
         <f>IF(AND($A8="",$C8="",$D8=""),"",IF($A8="","Missing QR Number",IF($C8="","Missing LastName",IF($D8="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A8,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A8,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -2648,53 +2660,53 @@
         <v>31</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="F9" s="12"/>
       <c r="G9" s="11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="J9" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="K9" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L9" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M9" s="12" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="N9" s="12" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="O9" s="12" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="P9" s="12" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="Q9" s="12" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="R9" s="12" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="S9" t="str">
         <f>IF(AND($A9="",$C9="",$D9=""),"",IF($A9="","Missing QR Number",IF($C9="","Missing LastName",IF($D9="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A9,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A9,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -2706,53 +2718,53 @@
         <v>31</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="F10" s="12"/>
       <c r="G10" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="I10" s="12" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="J10" s="11" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L10" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M10" s="12" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="N10" s="12" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="O10" s="12" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="P10" s="12" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="Q10" s="12" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="R10" s="12" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="S10" t="str">
         <f>IF(AND($A10="",$C10="",$D10=""),"",IF($A10="","Missing QR Number",IF($C10="","Missing LastName",IF($D10="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A10,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A10,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -2764,53 +2776,53 @@
         <v>32</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="F11" s="12"/>
       <c r="G11" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I11" s="12" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="J11" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="K11" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L11" s="12" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="M11" s="12" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="N11" s="12" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="O11" s="12" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="P11" s="12" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="Q11" s="12" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="R11" s="12" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="S11" t="str">
         <f>IF(AND($A11="",$C11="",$D11=""),"",IF($A11="","Missing QR Number",IF($C11="","Missing LastName",IF($D11="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A11,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A11,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -2822,53 +2834,53 @@
         <v>32</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="F12" s="12"/>
       <c r="G12" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="I12" s="12" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="J12" s="11" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K12" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L12" s="12" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="M12" s="12" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="N12" s="12" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="O12" s="12" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="P12" s="12" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="Q12" s="12" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="R12" s="12" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="S12" t="str">
         <f>IF(AND($A12="",$C12="",$D12=""),"",IF($A12="","Missing QR Number",IF($C12="","Missing LastName",IF($D12="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A12,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A12,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -2880,53 +2892,53 @@
         <v>33</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="F13" s="12"/>
       <c r="G13" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="I13" s="12" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="J13" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="K13" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L13" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M13" s="12" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="N13" s="12" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="O13" s="12" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="P13" s="12" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="Q13" s="12" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="R13" s="12" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="S13" t="str">
         <f>IF(AND($A13="",$C13="",$D13=""),"",IF($A13="","Missing QR Number",IF($C13="","Missing LastName",IF($D13="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A13,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A13,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -2938,49 +2950,49 @@
         <v>33</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="F14" s="12"/>
       <c r="G14" s="11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I14" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J14" s="11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="K14" s="12" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="L14" s="12" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="M14" s="12" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="N14" s="12" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="O14" s="12"/>
       <c r="P14" s="12"/>
       <c r="Q14" s="12" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="R14" s="12" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="S14" t="str">
         <f>IF(AND($A14="",$C14="",$D14=""),"",IF($A14="","Missing QR Number",IF($C14="","Missing LastName",IF($D14="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A14,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A14,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -2992,53 +3004,53 @@
         <v>34</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="F15" s="12"/>
       <c r="G15" s="11" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="I15" s="12" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="J15" s="11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K15" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L15" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M15" s="12" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="N15" s="12" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="O15" s="12" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="P15" s="12" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="Q15" s="12" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="R15" s="12" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="S15" t="str">
         <f>IF(AND($A15="",$C15="",$D15=""),"",IF($A15="","Missing QR Number",IF($C15="","Missing LastName",IF($D15="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A15,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A15,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -3050,53 +3062,53 @@
         <v>35</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="F16" s="12"/>
       <c r="G16" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H16" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I16" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K16" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L16" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M16" s="12" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="N16" s="12" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="O16" s="12" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="P16" s="12" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="Q16" s="12" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="R16" s="12" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="S16" t="str">
         <f>IF(AND($A16="",$C16="",$D16=""),"",IF($A16="","Missing QR Number",IF($C16="","Missing LastName",IF($D16="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A16,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A16,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -3108,53 +3120,53 @@
         <v>36</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F17" s="12"/>
       <c r="G17" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H17" s="12" t="s">
-        <v>138</v>
+        <v>215</v>
       </c>
       <c r="I17" s="12" t="s">
-        <v>139</v>
+        <v>217</v>
       </c>
       <c r="J17" s="11" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="K17" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L17" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M17" s="12" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="N17" s="12" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="O17" s="12" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="P17" s="12" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="Q17" s="12" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="R17" s="12" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="S17" t="str">
         <f>IF(AND($A17="",$C17="",$D17=""),"",IF($A17="","Missing QR Number",IF($C17="","Missing LastName",IF($D17="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A17,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A17,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -3166,53 +3178,53 @@
         <v>37</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="F18" s="12"/>
       <c r="G18" s="11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H18" s="12" t="s">
-        <v>211</v>
+        <v>141</v>
       </c>
       <c r="I18" s="12" t="s">
-        <v>213</v>
+        <v>142</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K18" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L18" s="12" t="s">
-        <v>141</v>
+        <v>227</v>
       </c>
       <c r="M18" s="12" t="s">
-        <v>142</v>
+        <v>232</v>
       </c>
       <c r="N18" s="12" t="s">
-        <v>143</v>
+        <v>242</v>
       </c>
       <c r="O18" s="12" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="P18" s="12" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="Q18" s="12" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="R18" s="12" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="S18" t="str">
         <f>IF(AND($A18="",$C18="",$D18=""),"",IF($A18="","Missing QR Number",IF($C18="","Missing LastName",IF($D18="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A18,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A18,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -3224,51 +3236,53 @@
         <v>38</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="E19" s="12"/>
+        <v>188</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>211</v>
+      </c>
       <c r="F19" s="12"/>
       <c r="G19" s="11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>138</v>
+        <v>215</v>
       </c>
       <c r="I19" s="12" t="s">
-        <v>139</v>
+        <v>217</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="K19" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L19" s="12" t="s">
-        <v>224</v>
+        <v>144</v>
       </c>
       <c r="M19" s="12" t="s">
-        <v>227</v>
+        <v>145</v>
       </c>
       <c r="N19" s="12" t="s">
-        <v>238</v>
+        <v>146</v>
       </c>
       <c r="O19" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="P19" s="12" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="Q19" s="12" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="R19" s="12" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="S19" t="str">
         <f>IF(AND($A19="",$C19="",$D19=""),"",IF($A19="","Missing QR Number",IF($C19="","Missing LastName",IF($D19="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A19,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A19,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -3280,55 +3294,55 @@
         <v>39</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="C20" s="12"/>
+        <v>137</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>163</v>
+      </c>
       <c r="D20" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="E20" s="12" t="s">
-        <v>202</v>
-      </c>
+        <v>189</v>
+      </c>
+      <c r="E20" s="12"/>
       <c r="F20" s="12"/>
       <c r="G20" s="11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>211</v>
+        <v>141</v>
       </c>
       <c r="I20" s="12" t="s">
-        <v>213</v>
+        <v>142</v>
       </c>
       <c r="J20" s="11" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="K20" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L20" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M20" s="12" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="N20" s="12" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="O20" s="12" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="P20" s="12" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="Q20" s="12" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="R20" s="12" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="S20" t="str">
         <f>IF(AND($A20="",$C20="",$D20=""),"",IF($A20="","Missing QR Number",IF($C20="","Missing LastName",IF($D20="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A20,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A20,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
-        <v>Missing LastName</v>
+        <v>More than one Head</v>
       </c>
     </row>
     <row r="21" spans="1:19">
@@ -3336,169 +3350,167 @@
         <v>40</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>160</v>
-      </c>
-      <c r="D21" s="12"/>
+        <v>137</v>
+      </c>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12" t="s">
+        <v>190</v>
+      </c>
       <c r="E21" s="12" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="F21" s="12"/>
       <c r="G21" s="11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H21" s="12" t="s">
-        <v>138</v>
+        <v>215</v>
       </c>
       <c r="I21" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J21" s="11" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="K21" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L21" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M21" s="12" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="N21" s="12" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="O21" s="12" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="P21" s="12" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="Q21" s="12" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="R21" s="12" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="S21" t="str">
         <f>IF(AND($A21="",$C21="",$D21=""),"",IF($A21="","Missing QR Number",IF($C21="","Missing LastName",IF($D21="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A21,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A21,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
-        <v>Missing FirstName</v>
+        <v>Missing LastName</v>
       </c>
     </row>
     <row r="22" spans="1:19">
-      <c r="A22" s="11"/>
+      <c r="A22" s="11" t="s">
+        <v>41</v>
+      </c>
       <c r="B22" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="D22" s="12" t="s">
-        <v>182</v>
-      </c>
+        <v>163</v>
+      </c>
+      <c r="D22" s="12"/>
       <c r="E22" s="12" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="F22" s="12"/>
       <c r="G22" s="11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I22" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J22" s="11" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="K22" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L22" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M22" s="12" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="N22" s="12" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="O22" s="12" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="P22" s="12" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="Q22" s="12" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="R22" s="12" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="S22" t="str">
         <f>IF(AND($A22="",$C22="",$D22=""),"",IF($A22="","Missing QR Number",IF($C22="","Missing LastName",IF($D22="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A22,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A22,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
-        <v>Missing QR Number</v>
+        <v>Missing FirstName</v>
       </c>
     </row>
     <row r="23" spans="1:19">
-      <c r="A23" s="11" t="s">
-        <v>41</v>
-      </c>
+      <c r="A23" s="11"/>
       <c r="B23" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F23" s="12"/>
       <c r="G23" s="11" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H23" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I23" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J23" s="11" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="K23" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L23" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M23" s="12" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="N23" s="12" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="O23" s="12" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="P23" s="12" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="Q23" s="12" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="R23" s="12" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="S23" t="str">
         <f>IF(AND($A23="",$C23="",$D23=""),"",IF($A23="","Missing QR Number",IF($C23="","Missing LastName",IF($D23="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A23,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A23,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
-        <v>More than one Head</v>
+        <v>Missing QR Number</v>
       </c>
     </row>
     <row r="24" spans="1:19">
@@ -3506,53 +3518,53 @@
         <v>42</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="F24" s="12"/>
       <c r="G24" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>211</v>
+        <v>141</v>
       </c>
       <c r="I24" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J24" s="11" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K24" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L24" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M24" s="12" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="N24" s="12" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="O24" s="12" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="P24" s="12" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="Q24" s="12" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="R24" s="12" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="S24" t="str">
         <f>IF(AND($A24="",$C24="",$D24=""),"",IF($A24="","Missing QR Number",IF($C24="","Missing LastName",IF($D24="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A24,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A24,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -3564,53 +3576,53 @@
         <v>43</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="F25" s="12"/>
       <c r="G25" s="11" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H25" s="12" t="s">
-        <v>138</v>
+        <v>215</v>
       </c>
       <c r="I25" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J25" s="11" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="K25" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L25" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M25" s="12" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="N25" s="12" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="O25" s="12" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="P25" s="12" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="Q25" s="12" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="R25" s="12" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="S25" t="str">
         <f>IF(AND($A25="",$C25="",$D25=""),"",IF($A25="","Missing QR Number",IF($C25="","Missing LastName",IF($D25="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A25,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A25,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -3622,175 +3634,173 @@
         <v>44</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="F26" s="12"/>
       <c r="G26" s="11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H26" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I26" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="K26" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L26" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M26" s="12" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="N26" s="12" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="O26" s="12" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="P26" s="12" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="Q26" s="12" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="R26" s="12" t="s">
-        <v>288</v>
-      </c>
-      <c r="S26" t="e">
+        <v>291</v>
+      </c>
+      <c r="S26" t="str">
         <f>IF(AND($A26="",$C26="",$D26=""),"",IF($A26="","Missing QR Number",IF($C26="","Missing LastName",IF($D26="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A26,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A26,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
-        <v>#REF!</v>
+        <v>More than one Head</v>
       </c>
     </row>
     <row r="27" spans="1:19">
-      <c r="A27" s="13" t="s">
+      <c r="A27" s="11" t="s">
         <v>45</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F27" s="12"/>
       <c r="G27" s="11" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H27" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="I27" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="J27" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="K27" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="L27" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="M27" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="N27" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="O27" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="P27" s="12" t="s">
+        <v>267</v>
+      </c>
+      <c r="Q27" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="R27" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="S27" t="e">
+        <f>IF(AND($A27="",$C27="",$D27=""),"",IF($A27="","Missing QR Number",IF($C27="","Missing LastName",IF($D27="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A27,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A27,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19">
+      <c r="A28" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>188</v>
+      </c>
+      <c r="E28" s="12" t="s">
         <v>211</v>
       </c>
-      <c r="I27" s="12" t="s">
-        <v>213</v>
-      </c>
-      <c r="J27" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="K27" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="L27" s="12" t="s">
-        <v>224</v>
-      </c>
-      <c r="M27" s="12" t="s">
-        <v>229</v>
-      </c>
-      <c r="N27" s="12" t="s">
-        <v>238</v>
-      </c>
-      <c r="O27" s="12" t="s">
-        <v>255</v>
-      </c>
-      <c r="P27" s="12" t="s">
-        <v>264</v>
-      </c>
-      <c r="Q27" s="12" t="s">
-        <v>276</v>
-      </c>
-      <c r="R27" s="12" t="s">
-        <v>285</v>
-      </c>
-      <c r="S27" t="str">
-        <f>IF(AND($A27="",$C27="",$D27=""),"",IF($A27="","Missing QR Number",IF($C27="","Missing LastName",IF($D27="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A27,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A27,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="28" spans="1:19">
-      <c r="A28" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="B28" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="C28" s="12" t="s">
-        <v>167</v>
-      </c>
-      <c r="D28" s="12" t="s">
-        <v>189</v>
-      </c>
-      <c r="E28" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="F28" s="12" t="s">
-        <v>210</v>
-      </c>
+      <c r="F28" s="12"/>
       <c r="G28" s="11" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>138</v>
+        <v>215</v>
       </c>
       <c r="I28" s="12" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="J28" s="11" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="K28" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L28" s="12" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="M28" s="12" t="s">
         <v>232</v>
       </c>
       <c r="N28" s="12" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="O28" s="12" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="P28" s="12" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="Q28" s="12" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="R28" s="12" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="S28" t="str">
         <f>IF(AND($A28="",$C28="",$D28=""),"",IF($A28="","Missing QR Number",IF($C28="","Missing LastName",IF($D28="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A28,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A28,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
-        <v>More than one Head</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="29" spans="1:19">
@@ -3798,51 +3808,55 @@
         <v>47</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="F29" s="12"/>
+        <v>138</v>
+      </c>
+      <c r="F29" s="12" t="s">
+        <v>214</v>
+      </c>
       <c r="G29" s="11" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H29" s="12" t="s">
-        <v>211</v>
+        <v>141</v>
       </c>
       <c r="I29" s="12" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="J29" s="11" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="K29" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L29" s="12" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="M29" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="N29" s="12"/>
+        <v>235</v>
+      </c>
+      <c r="N29" s="12" t="s">
+        <v>240</v>
+      </c>
       <c r="O29" s="12" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="P29" s="12" t="s">
-        <v>145</v>
+        <v>274</v>
       </c>
       <c r="Q29" s="12" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="R29" s="12" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="S29" t="str">
         <f>IF(AND($A29="",$C29="",$D29=""),"",IF($A29="","Missing QR Number",IF($C29="","Missing LastName",IF($D29="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A29,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A29,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -3854,51 +3868,51 @@
         <v>48</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>205</v>
+        <v>138</v>
       </c>
       <c r="F30" s="12"/>
       <c r="G30" s="11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H30" s="12" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="I30" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="K30" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L30" s="12" t="s">
-        <v>224</v>
-      </c>
-      <c r="M30" s="12"/>
-      <c r="N30" s="12" t="s">
-        <v>143</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="M30" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="N30" s="12"/>
       <c r="O30" s="12" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="P30" s="12" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="Q30" s="12" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="R30" s="12" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="S30" t="str">
         <f>IF(AND($A30="",$C30="",$D30=""),"",IF($A30="","Missing QR Number",IF($C30="","Missing LastName",IF($D30="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A30,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A30,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -3910,51 +3924,51 @@
         <v>49</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>198</v>
+        <v>209</v>
       </c>
       <c r="F31" s="12"/>
       <c r="G31" s="11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H31" s="12" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="I31" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="K31" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="L31" s="12"/>
-      <c r="M31" s="12" t="s">
-        <v>142</v>
-      </c>
+        <v>143</v>
+      </c>
+      <c r="L31" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="M31" s="12"/>
       <c r="N31" s="12" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="O31" s="12" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="P31" s="12" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="Q31" s="12" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="R31" s="12" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="S31" t="str">
         <f>IF(AND($A31="",$C31="",$D31=""),"",IF($A31="","Missing QR Number",IF($C31="","Missing LastName",IF($D31="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A31,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A31,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -3966,51 +3980,51 @@
         <v>50</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F32" s="12"/>
       <c r="G32" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H32" s="12" t="s">
-        <v>211</v>
-      </c>
-      <c r="I32" s="12"/>
+        <v>215</v>
+      </c>
+      <c r="I32" s="12" t="s">
+        <v>217</v>
+      </c>
       <c r="J32" s="11" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="K32" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="L32" s="12" t="s">
-        <v>224</v>
-      </c>
+        <v>143</v>
+      </c>
+      <c r="L32" s="12"/>
       <c r="M32" s="12" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="N32" s="12" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="O32" s="12" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="P32" s="12" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="Q32" s="12" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="R32" s="12" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="S32" t="str">
         <f>IF(AND($A32="",$C32="",$D32=""),"",IF($A32="","Missing QR Number",IF($C32="","Missing LastName",IF($D32="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A32,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A32,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -4022,51 +4036,51 @@
         <v>51</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F33" s="12"/>
       <c r="G33" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="H33" s="12"/>
-      <c r="I33" s="12" t="s">
-        <v>213</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="H33" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="I33" s="12"/>
       <c r="J33" s="11" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="K33" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L33" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M33" s="12" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="N33" s="12" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="O33" s="12" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="P33" s="12" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="Q33" s="12" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="R33" s="12" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="S33" t="str">
         <f>IF(AND($A33="",$C33="",$D33=""),"",IF($A33="","Missing QR Number",IF($C33="","Missing LastName",IF($D33="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A33,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A33,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -4078,51 +4092,51 @@
         <v>52</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="F34" s="12"/>
-      <c r="G34" s="11"/>
-      <c r="H34" s="12" t="s">
-        <v>211</v>
-      </c>
+      <c r="G34" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="H34" s="12"/>
       <c r="I34" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="K34" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L34" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M34" s="12" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="N34" s="12" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="O34" s="12" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="P34" s="12" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="Q34" s="12" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="R34" s="12" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="S34" t="str">
         <f>IF(AND($A34="",$C34="",$D34=""),"",IF($A34="","Missing QR Number",IF($C34="","Missing LastName",IF($D34="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A34,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A34,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -4134,53 +4148,51 @@
         <v>53</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F35" s="12"/>
-      <c r="G35" s="11" t="s">
-        <v>88</v>
-      </c>
+      <c r="G35" s="11"/>
       <c r="H35" s="12" t="s">
-        <v>138</v>
+        <v>215</v>
       </c>
       <c r="I35" s="12" t="s">
-        <v>139</v>
+        <v>217</v>
       </c>
       <c r="J35" s="11" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="K35" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L35" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M35" s="12" t="s">
-        <v>228</v>
+        <v>145</v>
       </c>
       <c r="N35" s="12" t="s">
-        <v>235</v>
+        <v>146</v>
       </c>
       <c r="O35" s="12" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="P35" s="12" t="s">
-        <v>272</v>
+        <v>148</v>
       </c>
       <c r="Q35" s="12" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="R35" s="12" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="S35" t="str">
         <f>IF(AND($A35="",$C35="",$D35=""),"",IF($A35="","Missing QR Number",IF($C35="","Missing LastName",IF($D35="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A35,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A35,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -4189,52 +4201,56 @@
     </row>
     <row r="36" spans="1:19">
       <c r="A36" s="11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="F36" s="12"/>
       <c r="G36" s="11" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H36" s="12" t="s">
-        <v>211</v>
+        <v>141</v>
       </c>
       <c r="I36" s="12" t="s">
-        <v>213</v>
+        <v>142</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="K36" s="12" t="s">
-        <v>217</v>
+        <v>143</v>
       </c>
       <c r="L36" s="12" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="M36" s="12" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="N36" s="12" t="s">
-        <v>234</v>
-      </c>
-      <c r="O36" s="12"/>
-      <c r="P36" s="12"/>
+        <v>238</v>
+      </c>
+      <c r="O36" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="P36" s="12" t="s">
+        <v>275</v>
+      </c>
       <c r="Q36" s="12" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="R36" s="12" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="S36" t="str">
         <f>IF(AND($A36="",$C36="",$D36=""),"",IF($A36="","Missing QR Number",IF($C36="","Missing LastName",IF($D36="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A36,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A36,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -4243,52 +4259,52 @@
     </row>
     <row r="37" spans="1:19">
       <c r="A37" s="11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="F37" s="12"/>
       <c r="G37" s="11" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H37" s="12" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="I37" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J37" s="11" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="K37" s="12" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="L37" s="12" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="M37" s="12" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="N37" s="12" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="O37" s="12"/>
       <c r="P37" s="12"/>
       <c r="Q37" s="12" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="R37" s="12" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="S37" t="str">
         <f>IF(AND($A37="",$C37="",$D37=""),"",IF($A37="","Missing QR Number",IF($C37="","Missing LastName",IF($D37="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A37,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A37,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -4300,53 +4316,49 @@
         <v>54</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F38" s="12"/>
       <c r="G38" s="11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H38" s="12" t="s">
-        <v>138</v>
+        <v>215</v>
       </c>
       <c r="I38" s="12" t="s">
-        <v>139</v>
+        <v>217</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K38" s="12" t="s">
-        <v>140</v>
+        <v>223</v>
       </c>
       <c r="L38" s="12" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="M38" s="12" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="N38" s="12" t="s">
-        <v>235</v>
-      </c>
-      <c r="O38" s="12" t="s">
-        <v>258</v>
-      </c>
-      <c r="P38" s="12" t="s">
-        <v>273</v>
-      </c>
+        <v>237</v>
+      </c>
+      <c r="O38" s="12"/>
+      <c r="P38" s="12"/>
       <c r="Q38" s="12" t="s">
-        <v>146</v>
+        <v>279</v>
       </c>
       <c r="R38" s="12" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="S38" t="str">
         <f>IF(AND($A38="",$C38="",$D38=""),"",IF($A38="","Missing QR Number",IF($C38="","Missing LastName",IF($D38="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A38,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A38,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -4358,53 +4370,53 @@
         <v>55</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F39" s="12"/>
       <c r="G39" s="11" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H39" s="12" t="s">
-        <v>211</v>
+        <v>141</v>
       </c>
       <c r="I39" s="12" t="s">
-        <v>213</v>
+        <v>142</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="K39" s="12" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L39" s="12" t="s">
-        <v>141</v>
+        <v>227</v>
       </c>
       <c r="M39" s="12" t="s">
-        <v>142</v>
+        <v>236</v>
       </c>
       <c r="N39" s="12" t="s">
-        <v>143</v>
+        <v>238</v>
       </c>
       <c r="O39" s="12" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="P39" s="12" t="s">
-        <v>263</v>
+        <v>276</v>
       </c>
       <c r="Q39" s="12" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="R39" s="12" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="S39" t="str">
         <f>IF(AND($A39="",$C39="",$D39=""),"",IF($A39="","Missing QR Number",IF($C39="","Missing LastName",IF($D39="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A39,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A39,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -4413,52 +4425,56 @@
     </row>
     <row r="40" spans="1:19">
       <c r="A40" s="11" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="F40" s="12"/>
       <c r="G40" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H40" s="12" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="I40" s="12" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K40" s="12" t="s">
-        <v>220</v>
+        <v>143</v>
       </c>
       <c r="L40" s="12" t="s">
-        <v>222</v>
+        <v>144</v>
       </c>
       <c r="M40" s="12" t="s">
-        <v>225</v>
+        <v>145</v>
       </c>
       <c r="N40" s="12" t="s">
-        <v>234</v>
-      </c>
-      <c r="O40" s="12"/>
-      <c r="P40" s="12"/>
+        <v>146</v>
+      </c>
+      <c r="O40" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="P40" s="12" t="s">
+        <v>266</v>
+      </c>
       <c r="Q40" s="12" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="R40" s="12" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="S40" t="str">
         <f>IF(AND($A40="",$C40="",$D40=""),"",IF($A40="","Missing QR Number",IF($C40="","Missing LastName",IF($D40="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A40,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A40,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -4467,56 +4483,52 @@
     </row>
     <row r="41" spans="1:19">
       <c r="A41" s="11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="E41" s="12" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="F41" s="12"/>
       <c r="G41" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H41" s="12" t="s">
-        <v>138</v>
+        <v>215</v>
       </c>
       <c r="I41" s="12" t="s">
-        <v>139</v>
+        <v>217</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="K41" s="12" t="s">
-        <v>140</v>
+        <v>224</v>
       </c>
       <c r="L41" s="12" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="M41" s="12" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="N41" s="12" t="s">
-        <v>235</v>
-      </c>
-      <c r="O41" s="12" t="s">
-        <v>260</v>
-      </c>
-      <c r="P41" s="12" t="s">
-        <v>274</v>
-      </c>
+        <v>237</v>
+      </c>
+      <c r="O41" s="12"/>
+      <c r="P41" s="12"/>
       <c r="Q41" s="12" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="R41" s="12" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="S41" t="str">
         <f>IF(AND($A41="",$C41="",$D41=""),"",IF($A41="","Missing QR Number",IF($C41="","Missing LastName",IF($D41="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A41,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A41,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
@@ -4524,79 +4536,113 @@
       </c>
     </row>
     <row r="42" spans="1:19">
-      <c r="A42" s="11"/>
+      <c r="A42" s="11" t="s">
+        <v>57</v>
+      </c>
       <c r="B42" s="12" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="E42" s="12" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="F42" s="12"/>
       <c r="G42" s="11" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H42" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I42" s="12" t="s">
-        <v>213</v>
+        <v>142</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="K42" s="12" t="s">
-        <v>221</v>
+        <v>143</v>
       </c>
       <c r="L42" s="12" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="M42" s="12" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="N42" s="12" t="s">
-        <v>234</v>
-      </c>
-      <c r="O42" s="12"/>
-      <c r="P42" s="12"/>
+        <v>238</v>
+      </c>
+      <c r="O42" s="12" t="s">
+        <v>263</v>
+      </c>
+      <c r="P42" s="12" t="s">
+        <v>277</v>
+      </c>
       <c r="Q42" s="12" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="R42" s="12" t="s">
-        <v>284</v>
+        <v>293</v>
       </c>
       <c r="S42" t="str">
         <f>IF(AND($A42="",$C42="",$D42=""),"",IF($A42="","Missing QR Number",IF($C42="","Missing LastName",IF($D42="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A42,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A42,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
-        <v>Missing QR Number</v>
+        <v>More than one Head</v>
       </c>
     </row>
     <row r="43" spans="1:19">
       <c r="A43" s="11"/>
-      <c r="B43" s="12"/>
-      <c r="C43" s="12"/>
-      <c r="D43" s="12"/>
-      <c r="E43" s="12"/>
+      <c r="B43" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="C43" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="D43" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="E43" s="12" t="s">
+        <v>204</v>
+      </c>
       <c r="F43" s="12"/>
-      <c r="G43" s="11"/>
-      <c r="H43" s="12"/>
-      <c r="I43" s="12"/>
-      <c r="J43" s="11"/>
-      <c r="K43" s="12"/>
-      <c r="L43" s="12"/>
-      <c r="M43" s="12"/>
-      <c r="N43" s="12"/>
+      <c r="G43" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="H43" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="I43" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="J43" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="K43" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="L43" s="12" t="s">
+        <v>225</v>
+      </c>
+      <c r="M43" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="N43" s="12" t="s">
+        <v>237</v>
+      </c>
       <c r="O43" s="12"/>
       <c r="P43" s="12"/>
-      <c r="Q43" s="12"/>
-      <c r="R43" s="12"/>
+      <c r="Q43" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="R43" s="12" t="s">
+        <v>287</v>
+      </c>
       <c r="S43" t="str">
         <f>IF(AND($A43="",$C43="",$D43=""),"",IF($A43="","Missing QR Number",IF($C43="","Missing LastName",IF($D43="","Missing FirstName",IF(COUNTIFS($A$3:$A$1000,$A43,$B$3:$B$1000,"Head")=0,"No Head in this family",IF(COUNTIFS($A$3:$A$1000,$A43,$B$3:$B$1000,"Head")&gt;1,"More than one Head","OK"))))))</f>
-        <v/>
+        <v>Missing QR Number</v>
       </c>
     </row>
     <row r="44" spans="1:19">
@@ -27575,7 +27621,7 @@
     <mergeCell ref="O1:P1"/>
     <mergeCell ref="Q1:Q1"/>
     <mergeCell ref="R1:R1"/>
-    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="A42:A43"/>
   </mergeCells>
   <conditionalFormatting sqref="S3:S1000">
     <cfRule type="expression" dxfId="0" priority="1">
@@ -27661,908 +27707,908 @@
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="J1" s="1"/>
       <c r="K1" s="1" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="M1" s="1"/>
       <c r="N1" s="1" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
     </row>
     <row r="2" spans="1:16">
       <c r="A2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B2" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="C2" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D2" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="E2" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="F2" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="G2" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="H2" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="I2" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="K2" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="L2" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="N2" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="O2" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="P2" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
     </row>
     <row r="3" spans="1:16">
       <c r="A3" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="B3" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="C3" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="D3" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="E3" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="F3" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="G3" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="H3" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="I3" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="K3" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="L3" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="N3" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="O3" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="P3" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
     </row>
     <row r="4" spans="1:16">
       <c r="A4" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="B4" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="D4" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="E4" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="F4" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="G4" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="H4" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="I4" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="K4" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="L4" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="N4" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="O4" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="P4" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
     </row>
     <row r="5" spans="1:16">
       <c r="A5" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="B5" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="D5" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="E5" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="F5" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="G5" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="H5" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="I5" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="K5" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="L5" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="N5" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="O5" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="P5" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
     </row>
     <row r="6" spans="1:16">
       <c r="A6" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B6" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="D6" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="E6" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="F6" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="G6" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="H6" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="I6" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="K6" t="s">
+        <v>396</v>
+      </c>
+      <c r="L6" t="s">
+        <v>397</v>
+      </c>
+      <c r="N6" t="s">
+        <v>417</v>
+      </c>
+      <c r="O6" t="s">
+        <v>418</v>
+      </c>
+      <c r="P6" t="s">
         <v>392</v>
-      </c>
-      <c r="L6" t="s">
-        <v>393</v>
-      </c>
-      <c r="N6" t="s">
-        <v>413</v>
-      </c>
-      <c r="O6" t="s">
-        <v>414</v>
-      </c>
-      <c r="P6" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="7" spans="1:16">
       <c r="A7" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="B7" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="D7" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="E7" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="F7" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="G7" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="H7" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="I7" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="K7" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="L7" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="N7" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="O7" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="P7" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
     </row>
     <row r="8" spans="1:16">
       <c r="A8" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B8" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="E8" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F8" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="G8" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="H8" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="I8" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="K8" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="L8" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="N8" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="O8" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="P8" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
     </row>
     <row r="9" spans="1:16">
       <c r="A9" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="E9" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="G9" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="H9" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="I9" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="K9" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="L9" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="N9" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="O9" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="P9" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
     </row>
     <row r="10" spans="1:16">
       <c r="A10" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="E10" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="G10" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="H10" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="I10" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="K10" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="L10" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="N10" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="O10" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="P10" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
     </row>
     <row r="11" spans="1:16">
       <c r="A11" t="s">
-        <v>281</v>
+        <v>303</v>
       </c>
       <c r="E11" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="G11" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="H11" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="I11" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="K11" t="s">
-        <v>281</v>
+        <v>303</v>
       </c>
       <c r="L11" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="N11" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="O11" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="P11" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
     </row>
     <row r="12" spans="1:16">
       <c r="E12" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="G12" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="H12" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="I12" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="K12" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="L12" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="N12" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="O12" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="P12" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
     </row>
     <row r="13" spans="1:16">
       <c r="E13" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="G13" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="I13" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="N13" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="O13" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="P13" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
     </row>
     <row r="14" spans="1:16">
       <c r="E14" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="G14" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="I14" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="N14" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="O14" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="P14" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
     </row>
     <row r="15" spans="1:16">
       <c r="G15" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="I15" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="N15" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="O15" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="P15" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
     </row>
     <row r="16" spans="1:16">
       <c r="G16" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="I16" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="N16" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="O16" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="P16" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
     </row>
     <row r="17" spans="1:16">
       <c r="G17" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="I17" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="N17" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="O17" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="P17" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
     </row>
     <row r="18" spans="1:16">
       <c r="I18" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="N18" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="O18" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="P18" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
     </row>
     <row r="19" spans="1:16">
       <c r="I19" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="N19" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="O19" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="P19" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
     </row>
     <row r="20" spans="1:16">
       <c r="I20" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="N20" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="O20" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="P20" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
     </row>
     <row r="21" spans="1:16">
       <c r="I21" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="N21" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="O21" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="P21" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
     </row>
     <row r="22" spans="1:16">
       <c r="I22" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="N22" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="O22" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="P22" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
     </row>
     <row r="23" spans="1:16">
       <c r="I23" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="N23" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="O23" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="P23" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
     </row>
     <row r="24" spans="1:16">
       <c r="I24" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="N24" t="s">
+        <v>452</v>
+      </c>
+      <c r="O24" t="s">
+        <v>422</v>
+      </c>
+      <c r="P24" t="s">
         <v>448</v>
-      </c>
-      <c r="O24" t="s">
-        <v>418</v>
-      </c>
-      <c r="P24" t="s">
-        <v>444</v>
       </c>
     </row>
     <row r="25" spans="1:16">
       <c r="I25" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="N25" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="O25" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="P25" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
     </row>
     <row r="26" spans="1:16">
       <c r="N26" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="O26" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="P26" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
     </row>
     <row r="27" spans="1:16">
       <c r="N27" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="O27" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="P27" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
     </row>
     <row r="28" spans="1:16">
       <c r="N28" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="O28" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="P28" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
     </row>
     <row r="29" spans="1:16">
       <c r="N29" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="O29" t="s">
+        <v>463</v>
+      </c>
+      <c r="P29" t="s">
         <v>459</v>
-      </c>
-      <c r="P29" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="30" spans="1:16">
       <c r="N30" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="O30" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="P30" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
     </row>
     <row r="31" spans="1:16">
       <c r="N31" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="O31" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="P31" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
     </row>
     <row r="32" spans="1:16">
       <c r="N32" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="O32" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="P32" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
     </row>
     <row r="33" spans="1:16">
       <c r="N33" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="O33" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="P33" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
     </row>
     <row r="34" spans="1:16">
       <c r="N34" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="O34" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="P34" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
     </row>
     <row r="35" spans="1:16">
       <c r="N35" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="O35" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="P35" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
     </row>
     <row r="36" spans="1:16">
       <c r="N36" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="O36" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="P36" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
     </row>
     <row r="37" spans="1:16">
       <c r="N37" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="O37" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="P37" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
     </row>
     <row r="38" spans="1:16">
       <c r="N38" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="O38" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="P38" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
     </row>
     <row r="39" spans="1:16">
       <c r="N39" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="O39" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="P39" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
     </row>
     <row r="40" spans="1:16">
       <c r="N40" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="O40" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="P40" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
     </row>
     <row r="41" spans="1:16">
       <c r="N41" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="O41" t="s">
+        <v>488</v>
+      </c>
+      <c r="P41" t="s">
         <v>484</v>
-      </c>
-      <c r="P41" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="42" spans="1:16">
       <c r="N42" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="O42" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="P42" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
     </row>
     <row r="43" spans="1:16">
       <c r="N43" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="O43" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="P43" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
     </row>
     <row r="44" spans="1:16">
       <c r="N44" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="O44" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="P44" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
     </row>
     <row r="45" spans="1:16">
       <c r="N45" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="O45" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="P45" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
     </row>
     <row r="46" spans="1:16">
       <c r="N46" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
       <c r="O46" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="P46" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
     </row>
     <row r="47" spans="1:16">
       <c r="N47" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="O47" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="P47" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
     </row>
   </sheetData>
@@ -28694,53 +28740,53 @@
         <v>26</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="F3" s="8"/>
       <c r="G3" s="8" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="O3" s="8" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="P3" s="8" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="Q3" s="8" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="R3" s="8" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -28748,49 +28794,49 @@
         <v>26</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F4" s="8"/>
       <c r="G4" s="8" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="O4" s="8"/>
       <c r="P4" s="8"/>
       <c r="Q4" s="8" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
     </row>
     <row r="5" spans="1:18">
@@ -28798,43 +28844,43 @@
         <v>26</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="F5" s="8"/>
       <c r="G5" s="8" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J5" s="8"/>
       <c r="K5" s="8"/>
       <c r="L5" s="8" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="M5" s="8" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="N5" s="8"/>
       <c r="O5" s="8"/>
       <c r="P5" s="8"/>
       <c r="Q5" s="8" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="R5" s="8" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
     </row>
     <row r="6" spans="1:18">
@@ -28842,56 +28888,56 @@
         <v>27</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
       <c r="G6" s="8" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="L6" s="8" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="M6" s="8" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="N6" s="8" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="O6" s="8" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="P6" s="8" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="Q6" s="8" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="R6" s="8" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
     </row>
     <row r="8" spans="1:18" customHeight="1" ht="70">
       <c r="A8" s="9" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
     </row>
   </sheetData>

</xml_diff>